<commit_message>
Journal: log 2026-09-15 session and the 23700 PE trend short
Daily Analysis, Signals, Paper Trades, Levels Worked, and Lessons Log
for 2026-09-15 — a strong trend-down day (open 23576 to close 23118.6).
Records the taken short: 23700 PE (0DTE) 235 -> 365, +Rs8,450, held the
trend off the 09:25 retest. Lessons on trend-day entry timing, VIX
under-sizing gap days, and watcher reliability.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading_Journal.xlsx
+++ b/Trading_Journal.xlsx
@@ -1715,15 +1715,31 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n"/>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="11" t="n"/>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>23118.6</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>23448</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>23231</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>23398.1</v>
+      </c>
       <c r="F7" s="11" t="n"/>
       <c r="G7" s="11" t="n"/>
-      <c r="H7" s="11" t="n"/>
-      <c r="I7" s="11" t="n"/>
+      <c r="H7" s="11" t="n">
+        <v>23319</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <v>23435</v>
+      </c>
       <c r="J7" s="11" t="n"/>
       <c r="K7" s="11" t="n"/>
       <c r="L7" s="11" t="n"/>
@@ -1734,11 +1750,29 @@
       <c r="N7" s="11" t="n"/>
       <c r="O7" s="11" t="n"/>
       <c r="P7" s="11" t="n"/>
-      <c r="Q7" s="11" t="n"/>
-      <c r="R7" s="11" t="n"/>
-      <c r="S7" s="11" t="n"/>
-      <c r="T7" s="11" t="n"/>
-      <c r="U7" s="11" t="n"/>
+      <c r="Q7" s="11" t="inlineStr">
+        <is>
+          <t>Normal (VIX 12.29) - but range blew past it</t>
+        </is>
+      </c>
+      <c r="R7" s="11" t="inlineStr">
+        <is>
+          <t>1 SHORT taken - WIN +Rs8,450</t>
+        </is>
+      </c>
+      <c r="S7" s="11" t="n">
+        <v>85</v>
+      </c>
+      <c r="T7" s="11" t="inlineStr">
+        <is>
+          <t>NIFTY 2026-09-15 23700 PE</t>
+        </is>
+      </c>
+      <c r="U7" s="11" t="inlineStr">
+        <is>
+          <t>Gap UP +178 to 23576, tagged 23592 then RELENTLESS one-way sell - closed AT the low 23118.6 (range 474pts, far beyond VIX ~150-200). Flips all SHORT and correct. TRADE TAKEN: shorted the 09:25 retest (23500) via 23700 PE deep-ITM, held the trend to 12:30 = +Rs8,450 (235-&gt;365). Being at the screen for the retest is what captured it - the confirm-relay loop alone would have been ~20pts late. Levels gave reactions (23374/23319/23294/23263 rejects) but none held - trend day.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="n"/>
@@ -3939,21 +3973,65 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="n"/>
-      <c r="B5" s="20" t="n"/>
-      <c r="C5" s="20" t="n"/>
-      <c r="D5" s="20" t="n"/>
-      <c r="E5" s="20" t="n"/>
-      <c r="F5" s="20" t="n"/>
-      <c r="G5" s="20" t="n"/>
-      <c r="H5" s="20" t="n"/>
-      <c r="I5" s="20" t="n"/>
-      <c r="J5" s="20" t="n"/>
-      <c r="K5" s="20" t="n"/>
-      <c r="L5" s="20" t="n"/>
-      <c r="M5" s="20" t="n"/>
-      <c r="N5" s="20" t="n"/>
-      <c r="O5" s="20" t="n"/>
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>09:25</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>NIFTY</t>
+        </is>
+      </c>
+      <c r="D5" s="20" t="inlineStr">
+        <is>
+          <t>NIFTY 2026-09-15 23700 PE</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="F5" s="20" t="n">
+        <v>235</v>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>85</v>
+      </c>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>ITM (deep)</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J5" s="20" t="n">
+        <v>23500</v>
+      </c>
+      <c r="K5" s="20" t="n">
+        <v>23525</v>
+      </c>
+      <c r="L5" s="20" t="n">
+        <v>23460</v>
+      </c>
+      <c r="M5" s="20" t="n">
+        <v>23435</v>
+      </c>
+      <c r="N5" s="20" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="O5" s="20" t="inlineStr">
+        <is>
+          <t>CONFIRMED SHORT flip (23500 broke, retest rejected). TAKEN 09:25 as app capture via 23700 PE (deep ITM). Held the trend to 12:30, 235-&gt;365 = +Rs8,450. See Paper Trades.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n"/>
@@ -5921,7 +5999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="12" customWidth="1" style="36" min="1" max="1"/>
@@ -6241,6 +6319,118 @@
       <c r="F11" s="30" t="inlineStr">
         <is>
           <t>WORKED (magic, traded)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>23319</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>97</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Most-tested level of the day (21 tests, 8 rejects) - the afternoon base, but the trend eventually broke it too.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Reacted, did not hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>23374</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>88</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>3 rejects on the way down, slowed the fall but broke.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Reacted, did not hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>23294</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>86</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4 rejects near the lows; bounce attempts failed as the trend continued.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Reacted, did not hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>23263</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>84</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2 rejects; held briefly then gave way into the 23118 close.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Reacted, did not hold</t>
         </is>
       </c>
     </row>
@@ -7256,20 +7446,46 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n"/>
-      <c r="B5" s="11" t="n"/>
-      <c r="C5" s="11" t="n"/>
-      <c r="D5" s="11" t="n"/>
-      <c r="E5" s="11" t="n"/>
-      <c r="F5" s="11" t="n"/>
-      <c r="G5" s="11" t="n"/>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>NIFTY 2026-09-15 23700 PE</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>235</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>180</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>275</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>320</v>
+      </c>
       <c r="H5" s="15">
         <f>IFERROR((F5-D5)/(D5-E5),"")</f>
         <v/>
       </c>
-      <c r="I5" s="11" t="n"/>
-      <c r="J5" s="11" t="n"/>
-      <c r="K5" s="11" t="n"/>
+      <c r="I5" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>65</v>
+      </c>
+      <c r="K5" s="11" t="n">
+        <v>365</v>
+      </c>
       <c r="L5" s="16">
         <f>IF(OR(K5="",D5="",J5=""),"",(K5-D5)*J5)</f>
         <v/>
@@ -7279,7 +7495,11 @@
         <v/>
       </c>
       <c r="N5" s="11" t="n"/>
-      <c r="O5" s="11" t="n"/>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>SHORT flip (trend day). Captured on app 09:25 at the 23500 retest, deep-ITM PE (~0.95 delta). HELD the trend (not bank-half) to 12:30, exit 365 = +130 pts = +Rs8,450/lot. Rode the one-way sell 23470-&gt;23330.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="n"/>
@@ -10599,25 +10819,85 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Trend day</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Strong trend-down day (open 23576 -&gt; close AT low 23118). The flip shorts confirmed ~20pts late via the relay loop, BUT being at the screen the 09:25 retest was shorted live via a deep-ITM 23700 PE and HELD the trend to 12:30 = +Rs8,450.</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Proves the fix: on a trend day, entering at the retest LIVE (not waiting for the relay) captures the move. A deep-ITM PE (~0.95 delta) tracked the fall nearly 1:1 - good vehicle for a strong trend.</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>On a clear trend day: enter at the level-retest as it happens; consider a deep-ITM option for ~1:1 tracking; HOLD the trend (trail) rather than banking a fixed +40.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>VIX 12.29 predicted a ~150-200 pt day; actual range was 474 pts (2.5x). A gap-up + trend blew far past the VIX window, and the anchored +/-180 ladder left the watcher 'off the levels' below 23396 (had to widen to +/-400).</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>The VIX-scaled window under-sizes gap/trend days. Anchoring the ladder to only +/-VIX-window can leave you blind when price trends hard.</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>On a gap day, build the level ladder wider (&gt;= +/-400) from the start so a trend never runs off the map. Treat a big gap as a trend-risk day, not a range day.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Reliability</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>The watcher (scratchpad polling loop) slept twice today (missed ~10:00-12:24 and 12:31-close), losing most of the afternoon.</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Depending on my polling loop staying awake is fragile - a sleeping machine = no alerts for hours.</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Use a keep-awake for the session, and/or move the 5-min watch runner in-app so alerts do not depend on my polling.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n"/>

</xml_diff>